<commit_message>
Add Math, Physics, and Chemistry Equation Syntax Guide & Template integration
</commit_message>
<xml_diff>
--- a/Global_Questions_Master_Template.xlsx
+++ b/Global_Questions_Master_Template.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Physics_Examples" sheetId="4" r:id="rId4"/>
     <sheet name="Biology_Examples" sheetId="5" r:id="rId5"/>
     <sheet name="Instructions_Guide" sheetId="6" r:id="rId6"/>
+    <sheet name="Equations_Syntax_Guide" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -3195,4 +3196,338 @@
     <ignoredError numberStoredAsText="1" sqref="A1:C16"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E19"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Subject</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Concept</v>
+      </c>
+      <c r="C1" t="str">
+        <v>LaTeX Syntax</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Plain Unicode</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Example</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Mathematics</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Quadratic Formula</v>
+      </c>
+      <c r="C2" t="str">
+        <v>$x = \frac{-b \pm \sqrt{b^2 - 4ac}}{2a}$</v>
+      </c>
+      <c r="D2" t="str">
+        <v>x = (-b ± √(b² - 4ac)) / (2a)</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Solve $x^2 - 5x + 6 = 0$ using $x = \frac{-b \pm \sqrt{b^2 - 4ac}}{2a}$</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Mathematics</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Fractions</v>
+      </c>
+      <c r="C3" t="str">
+        <v>$\frac{numerator}{denominator}$</v>
+      </c>
+      <c r="D3" t="str">
+        <v>a / b</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Evaluate $\frac{2x + 1}{3} = 5$</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Mathematics</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Powers / Exponents</v>
+      </c>
+      <c r="C4" t="str">
+        <v>$x^2 + y^3 = z^n$</v>
+      </c>
+      <c r="D4" t="str">
+        <v>x² + y³ = zⁿ</v>
+      </c>
+      <c r="E4" t="str">
+        <v>If $2^{x+1} = 32$, find $x$.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Mathematics</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Square Root &amp; Radicals</v>
+      </c>
+      <c r="C5" t="str">
+        <v>$\sqrt{x}$ or $\sqrt[3]{27}$</v>
+      </c>
+      <c r="D5" t="str">
+        <v>√x or ∛27</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Simplify $\sqrt{75} + \sqrt{108}$</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Mathematics</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2x2 Matrix</v>
+      </c>
+      <c r="C6" t="str">
+        <v>$\begin{bmatrix} a &amp; b \\ c &amp; d \end{bmatrix}$</v>
+      </c>
+      <c r="D6" t="str">
+        <v>[[a, b], [c, d]]</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Find $|A|$ for $A = \begin{bmatrix} 2 &amp; -3 \\ 1 &amp; 4 \end{bmatrix}$</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Mathematics</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Trigonometry</v>
+      </c>
+      <c r="C7" t="str">
+        <v>$\sin^2\theta + \cos^2\theta = 1$</v>
+      </c>
+      <c r="D7" t="str">
+        <v>sin²θ + cos²θ = 1</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Prove $\tan\theta = \frac{\sin\theta}{\cos\theta}$</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Mathematics</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Sets &amp; Logic</v>
+      </c>
+      <c r="C8" t="str">
+        <v>$A \cup B$, $A \cap B$, $A'$</v>
+      </c>
+      <c r="D8" t="str">
+        <v>A ∪ B, A ∩ B, A'</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Verify $(A \cup B)' = A' \cap B'$</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Chemistry</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Chemical Formula</v>
+      </c>
+      <c r="C9" t="str">
+        <v>$\ce{H2SO4}$ or $\ce{C6H12O6}$</v>
+      </c>
+      <c r="D9" t="str">
+        <v>H₂SO₄ or C₆H₁₂O₆</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Molar mass of $\ce{H2SO4}$</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Chemistry</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Chemical Reactions</v>
+      </c>
+      <c r="C10" t="str">
+        <v>$\ce{2H2 + O2 -&gt; 2H2O}$</v>
+      </c>
+      <c r="D10" t="str">
+        <v>2H₂ + O₂ → 2H₂O</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Balance $\ce{CH4 + 2O2 -&gt; CO2 + 2H2O}$</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Chemistry</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Reversible Reaction</v>
+      </c>
+      <c r="C11" t="str">
+        <v>$\ce{N2 + 3H2 &lt;=&gt; 2NH3}$</v>
+      </c>
+      <c r="D11" t="str">
+        <v>N₂ + 3H₂ ⇌ 2NH₃</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Write $K_c$ for $\ce{N2 + 3H2 &lt;=&gt; 2NH3}$</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Chemistry</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Ions &amp; Charges</v>
+      </c>
+      <c r="C12" t="str">
+        <v>$\ce{Na+ + Cl- -&gt; NaCl}$ or $\ce{SO4^{2-}}$</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Na⁺ + Cl⁻ → NaCl</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Oxidation state of sulfur in $\ce{SO4^{2-}}$</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Chemistry</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Reaction Conditions (Heat)</v>
+      </c>
+      <c r="C13" t="str">
+        <v>$\ce{CaCO3 -&gt;[\Delta] CaO + CO2 ^}$</v>
+      </c>
+      <c r="D13" t="str">
+        <v>CaCO₃ →(heat) CaO + CO₂↑</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Decomposition of $\ce{CaCO3}$ under heat $\Delta$</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Physics</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Newton's 2nd Law</v>
+      </c>
+      <c r="C14" t="str">
+        <v>$F = ma$ or $\vec{F} = m\vec{a}$</v>
+      </c>
+      <c r="D14" t="str">
+        <v>F = ma (N = kg·m/s²)</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Force required for $m=1000\text{ kg}, a=2.5\text{ m/s}^2$</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Physics</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2nd Equation of Motion</v>
+      </c>
+      <c r="C15" t="str">
+        <v>$S = v_i t + \frac{1}{2}at^2$</v>
+      </c>
+      <c r="D15" t="str">
+        <v>S = vi·t + 0.5·a·t²</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Derive $S = v_i t + \frac{1}{2}at^2$</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Physics</v>
+      </c>
+      <c r="B16" t="str">
+        <v>3rd Equation of Motion</v>
+      </c>
+      <c r="C16" t="str">
+        <v>$2aS = v_f^2 - v_i^2$</v>
+      </c>
+      <c r="D16" t="str">
+        <v>2aS = vf² - vi²</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Calculate acceleration using $2aS = v_f^2 - v_i^2$</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Physics</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Kinetic Energy</v>
+      </c>
+      <c r="C17" t="str">
+        <v>$E_k = \frac{1}{2}mv^2$</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Ek = 1/2·m·v²</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Kinetic energy of $2\text{ kg}$ object at $10\text{ m/s}$</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Physics</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Ohm's Law &amp; Power</v>
+      </c>
+      <c r="C18" t="str">
+        <v>$V = IR$ and $P = \frac{V^2}{R}$</v>
+      </c>
+      <c r="D18" t="str">
+        <v>V = IR and P = V²/R</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Find resistance using $R = \frac{V^2}{P}$</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Physics</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Waves &amp; Time Period</v>
+      </c>
+      <c r="C19" t="str">
+        <v>$v = f\lambda$ and $T = 2\pi\sqrt{\frac{l}{g}}$</v>
+      </c>
+      <c r="D19" t="str">
+        <v>v = f·λ and T = 2π√(l/g)</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Time period of pendulum of length $1\text{ m}$</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E19"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>